<commit_message>
adjusted for PR discussions
</commit_message>
<xml_diff>
--- a/rules/CORE-000580/positive/03/data/unit-test-coreid-CG0325-positive03.xlsx
+++ b/rules/CORE-000580/positive/03/data/unit-test-coreid-CG0325-positive03.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\verisian\core-contributor\rules\CORE-000580\positive\03\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7930FADE-9DBF-41AA-B2DE-D415602496B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{782870FF-7FA5-4638-8B61-927EDDC0C1D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="43">
   <si>
     <t>Product</t>
   </si>
@@ -151,18 +151,6 @@
   </si>
   <si>
     <t>Z</t>
-  </si>
-  <si>
-    <t>TEENRL</t>
-  </si>
-  <si>
-    <t>Rule for End of Element</t>
-  </si>
-  <si>
-    <t>END OF TREATMENT1</t>
-  </si>
-  <si>
-    <t>END OF TREATMENT2</t>
   </si>
 </sst>
 </file>
@@ -613,10 +601,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr defaultColWidth="19" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
@@ -633,13 +621,10 @@
         <v>12</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="G1" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>14</v>
       </c>
@@ -656,13 +641,10 @@
         <v>18</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="G2" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>20</v>
       </c>
@@ -681,11 +663,8 @@
       <c r="F3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>10</v>
       </c>
@@ -702,13 +681,10 @@
         <v>51</v>
       </c>
       <c r="F4" s="3">
-        <v>51</v>
-      </c>
-      <c r="G4" s="3">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="120" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>21</v>
       </c>
@@ -724,11 +700,11 @@
       <c r="E5" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>21</v>
       </c>
@@ -745,13 +721,10 @@
         <v>29</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="G6" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>21</v>
       </c>
@@ -768,13 +741,10 @@
         <v>29</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="G7" s="4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="120" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>21</v>
       </c>
@@ -790,11 +760,11 @@
       <c r="E8" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="F8" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="120" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>21</v>
       </c>
@@ -810,11 +780,11 @@
       <c r="E9" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="F9" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>21</v>
       </c>
@@ -830,11 +800,11 @@
       <c r="E10" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="F10" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>21</v>
       </c>
@@ -850,11 +820,11 @@
       <c r="E11" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="F11" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>21</v>
       </c>
@@ -870,7 +840,7 @@
       <c r="E12" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="F12" s="5" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>